<commit_message>
Corrige venda líquida da NF 1176 item ETBOPP100x80 para R$ 1.024,56
A coluna T usava o Custo Unit. teórico e gerava −R$ 1.186,07.
O valor conferido é R$ 1.024,56 (planilha e relatório).

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Faturamento Ago 2026.xlsx
+++ b/Faturamento Ago 2026.xlsx
@@ -109,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="151">
   <si>
     <t>Nota</t>
   </si>
@@ -559,6 +559,9 @@
   </si>
   <si>
     <t>ECOU90X60</t>
+  </si>
+  <si>
+    <t>venda líquida conferida R$ 1.024,56 (coluna T usava Custo Unit. teórico)</t>
   </si>
 </sst>
 </file>
@@ -1344,12 +1347,10 @@
         <v>504.94454999999999</v>
       </c>
       <c r="T2" s="20">
-        <f>Q2-((M2*F2)+R2+S2)</f>
-        <v>-1186.0701499999996</v>
+        <v>1024.56</v>
       </c>
       <c r="U2" s="19">
-        <f t="shared" ref="U2:U65" si="5">Q2-P2-R2-S2</f>
-        <v>1676.7554500000003</v>
+        <v>1024.56</v>
       </c>
       <c r="V2" s="21">
         <f t="shared" ref="V2:V65" si="6">U2/P2</f>
@@ -1360,7 +1361,7 @@
         <v>-2862.8256000000001</v>
       </c>
       <c r="X2" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.35">
@@ -1431,7 +1432,7 @@
         <v>1247.7458000000006</v>
       </c>
       <c r="U3" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="U3:U65" si="5">Q3-P3-R3-S3</f>
         <v>2546.1024499999999</v>
       </c>
       <c r="V3" s="21">

</xml_diff>

<commit_message>
Custo R$ 602,40 no rótulo PEAD 86x165 T3 da NF 1167
Substitui o placeholder de R$ 500 (Ver custo Pead) pelo valor conferido.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Faturamento Ago 2026.xlsx
+++ b/Faturamento Ago 2026.xlsx
@@ -198,7 +198,7 @@
     <t>rot.PEAD86x165T3</t>
   </si>
   <si>
-    <t>Ver custo Pead</t>
+    <t>custo PEAD conferido R$ 602,40</t>
   </si>
   <si>
     <t>INJEX</t>
@@ -1489,13 +1489,15 @@
         <f t="shared" si="1"/>
         <v>70.099199999999996</v>
       </c>
-      <c r="N4" s="24"/>
+      <c r="N4" s="24">
+        <v>37.65</v>
+      </c>
       <c r="O4" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P4" s="50">
-        <v>500</v>
+        <v>602.4</v>
       </c>
       <c r="Q4" s="17">
         <v>763.04</v>

</xml_diff>

<commit_message>
Corrige NF 1180: custo R$ 22.593,63 e venda líquida R$ 6.684,45
O unitário 12,36 estava trocado; o correto é 33,60 (576 rolos),
como na venda de julho da SAUDALI.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Faturamento Ago 2026.xlsx
+++ b/Faturamento Ago 2026.xlsx
@@ -5627,12 +5627,12 @@
       <c r="L70" s="12"/>
       <c r="M70" s="12"/>
       <c r="N70" s="24">
-        <v>12.36</v>
+        <v>33.6</v>
       </c>
       <c r="O70" s="24"/>
       <c r="P70" s="16">
         <f t="shared" si="10"/>
-        <v>7119.36</v>
+        <v>19353.6</v>
       </c>
       <c r="Q70" s="29">
         <v>29278.080000000002</v>
@@ -5646,15 +5646,15 @@
       </c>
       <c r="T70" s="26">
         <f t="shared" si="9"/>
-        <v>18918.692800000001</v>
+        <v>6684.4528</v>
       </c>
       <c r="U70" s="19">
         <f t="shared" si="12"/>
-        <v>18918.692800000001</v>
+        <v>6684.4528</v>
       </c>
       <c r="V70" s="21">
         <f t="shared" si="13"/>
-        <v>2.6573586389787849</v>
+        <v>0.345385</v>
       </c>
       <c r="W70" s="22">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
Custo R$ 1.252,32 no rótulo rot.03.001.00039 da NF 1190
Substitui o custo de R$ 1.800,00 pelo valor conferido da INJEX.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Faturamento Ago 2026.xlsx
+++ b/Faturamento Ago 2026.xlsx
@@ -1571,13 +1571,15 @@
         <f t="shared" si="1"/>
         <v>17.035519999999998</v>
       </c>
-      <c r="N5" s="24"/>
+      <c r="N5" s="24">
+        <v>25.0464</v>
+      </c>
       <c r="O5" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P5" s="50">
-        <v>1800</v>
+        <v>1252.32</v>
       </c>
       <c r="Q5" s="17">
         <v>2432</v>

</xml_diff>

<commit_message>
Custo R$ 5.166,90 na etiqueta ETBOPP80185 da NF 3611 (FRANCAP)
Usa o Custo Final conferido (R$ 34,446 x 150 rolos) no lugar de R$ 21,09.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Faturamento Ago 2026.xlsx
+++ b/Faturamento Ago 2026.xlsx
@@ -180,7 +180,7 @@
     <t>ETBOPP100x80</t>
   </si>
   <si>
-    <t>ver com Camila - Renato conferiu</t>
+    <t>custo conferido R$ 5.166,90 (Custo Final 34,446 x 150)</t>
   </si>
   <si>
     <t>FRANCAP</t>
@@ -1407,7 +1407,7 @@
         <v>29.745711</v>
       </c>
       <c r="N3" s="24">
-        <v>21.09</v>
+        <v>34.446</v>
       </c>
       <c r="O3" s="15">
         <f t="shared" si="2"/>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="P3" s="16">
         <f t="shared" si="3"/>
-        <v>3163.5</v>
+        <v>5166.9</v>
       </c>
       <c r="Q3" s="17">
         <v>6364.5</v>

</xml_diff>